<commit_message>
Agregué casos de prueba para formato de contraseña incorrecto
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="92">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -241,6 +241,320 @@
       </rPr>
       <t xml:space="preserve">. No permite seleccionar la opción “Siguiente”.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">cp7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro con contraseña sin número</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: abcdefg$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechaza el formato de contraseña sin números</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro con contraseña sin caracteres especiales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: a2345678</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechaza el formato de contraseña sin caracteres especiales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error contraseña 1er intento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">usuario registrado en estado logged out</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123**</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Ingresar al sitio; 2- Seleccionar la opción “Regístrate en TikTok” con la opción correo electrónico; 3- Completar Email; 4- Completar contraseña; 5- seleccionar la opción “Iniciar sesión”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aviso de contraseña incorrecta sin pasar al estado blocked out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualiza la leyenda “Cuenta o contraseña incorrecta”, permitiendo otro intento para iniciar sesión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error contraseña 2do intento</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1- Ingresar al sitio; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2- Seleccionar la opción “Regístrate en TikTok” con la opción correo electrónico</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; 3- Completar Email; 4- Completar contraseña; 5- seleccionar la opción “Iniciar sesión” (x2)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualiza la leyenda “Cuenta o contraseña incorrecta. Quedan 5 intentos. Prueba otra vez”, permitiendo otro intento para iniciar sesión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error contraseña supera número máximo de intentos (7)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1- Ingresar al sitio; 2- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2- Seleccionar la opción “Regístrate en TikTok” con la opción correo electrónico</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; 3- Completar Email; 4- Completar contraseña; 5- seleccionar la opción “Iniciar sesión” (x8)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Aviso de contraseña incorrecta. El usuario pasa al estado blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se visualiza la leyenda “Has superado el límite de intentos para introducir la cuenta o la contraseña. Inténtalo de nuevo en 30 mm.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A medida que se realizan los intentos fallidos, se visualiza una cuenta regresiva que indica la cantidad de intentos restantes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inicio de sesión de usuario en estado blocked antes de completar el tiempo de espera para nuevos intentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">usuario en estado blocked</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1- Ingresar al sitio; 2-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Seleccionar la opción “Regístrate en TikTok” con la opción correo electrónico</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; 3- Completar Email; 4- Completar contraseña; 5- seleccionar la opción “Iniciar sesión” (x8); 6- seleccionar “Iniciar sesión” nuevamente</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario se mantiene en estado blocked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">se visualiza la leyenda “Has superado el límite de intentos para introducir la cuenta o la contraseña. Inténtalo de nuevo en 27 mm.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A medida que se realizan los intentos fallidos, se visualiza una cuenta regresiva que indica la cantidad de minutos restantes para volver a intentarlo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restablecer contraseña</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email: breru.qatest@gmail.com</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1- Ingresar al sitio; 2-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Seleccionar la opción “Regístrate en TikTok” con la opción correo electrónico</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; 3- Completar Email; 4- Seleccionar la opción “Siguiente”; 5- Seleccionar la opción “¿Olvidaste la contraseña?”; 6- Seleccionar la opción “Correo electrónico”; 7- Seleccionar la opción “Restablecer”</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario recibe un email con la información para recuperar la cuenta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La app envía un correo electrónico con un código numérico que expira luego de las 48hs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al ingresar el código, redirige a una nueva pantalla para crear una nueva contraseña con los requerimientos de seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error por ingreso de contraseña anterior al momento de crear una contraseña nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usuario registrado</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1- Ingresar al sitio; 2-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Seleccionar la opción “Regístrate en TikTok” con la opción correo electrónico</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">; 3- Completar Email; 4- Seleccionar la opción “Siguiente”; 5- Seleccionar la opción “¿Olvidaste la contraseña?”; 6- Seleccionar la opción “Correo electrónico”; 7- Seleccionar la opción “Restablecer”; 8- Ingresar código enviado por email; 9- Ingresar contraseña</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema rechaza la contraseña ingresada y solicita el ingreso de una contraseña nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualiza la leyenda “Tu nueva contraseña no puede ser la misma que la anterior”</t>
   </si>
 </sst>
 </file>
@@ -757,14 +1071,28 @@
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+    <row r="8" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -772,14 +1100,28 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+    <row r="9" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -787,14 +1129,28 @@
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+    <row r="10" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -802,14 +1158,28 @@
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+    <row r="11" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -817,59 +1187,121 @@
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+    <row r="12" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
+      <c r="K12" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+    <row r="13" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="K13" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+    <row r="14" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
+      <c r="K14" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+    <row r="15" customFormat="false" ht="184.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -878,13 +1310,8 @@
       <c r="M15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -1123,6 +1550,14 @@
     <hyperlink ref="D5" r:id="rId3" display="ejemplo@prueba.com"/>
     <hyperlink ref="D6" r:id="rId4" display="ejemplo@prueba.com"/>
     <hyperlink ref="D7" r:id="rId5" display="ejemplo@prueba.com"/>
+    <hyperlink ref="D8" r:id="rId6" display="ejemplo@prueba.com"/>
+    <hyperlink ref="D9" r:id="rId7" display="ejemplo@prueba.com"/>
+    <hyperlink ref="D10" r:id="rId8" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D11" r:id="rId9" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D12" r:id="rId10" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D13" r:id="rId11" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D14" r:id="rId12" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D15" r:id="rId13" display="breru.qatest@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1131,6 +1566,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId6"/>
+  <legacyDrawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Agregué casos de prueba de usabilidad / UX
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="129">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -555,6 +555,117 @@
   </si>
   <si>
     <t xml:space="preserve">Se visualiza la leyenda “Tu nueva contraseña no puede ser la misma que la anterior”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compartir video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">usuario en estado logged in </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Compartir” (símbolo flecha); 4- Seleccionar la aplicación WhatsApp; 5- Seleccionar un contacto; 6- Enviar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">el sistema permite compartir el video en diferentes redes sociales, entre ella WhatsApp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualizan los íconos de las diferentes aplicaciones a las que se puede compartir el contenido. Permite seleccionar contactos y enviar por WhatsApp </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dejar comentarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Comentar” (símbolo globo de diálogo); 4- Ingresar un comentario en el campo “Añadir comentario”; 5- Enviar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">el sistema permite añadir un comentario a la publicación seleccionada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al ingresar a los comentarios, se visualiza el último comentario agregado primero en la lista (orden: intercalados entre sí, con diferentes tiempos de realización)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al actualizar la pantalla e ingresar nuevamente al listado de comentarios de la publicación, cambia el orden de la lista. El último comentario realizado aparece al final (orden: del más antiguo al menos antiguo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">guardar contenido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Guardar” (símbolo de marcador); 4- Ingresar al perfil de usuario; 5- seleccionar mismo símbolo de marcador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualiza el contenido guardado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario accede a la vista previa de cada uno de los videos guardados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">visualizar Likes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Me gusta” (símbolo de corazón); 4- Ingresar al perfil de usuario; 5- seleccionar mismo símbolo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">se visualiza el contenido “likeado”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario accede a la vista previa de cada uno de los videos a los que le dio Like</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">crear contenido privado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- seleccionar la opción “Nuevo video” (símbolo “+”); 4- Seleccionar Cámara; 5- Crear publicación; 6- Seleccionar “Siguiente”; 7- Cambiar el ajuste de privacidad a “Sólo yo”; 8- Publicar; 9- Ingresar nuevamente al perfil; 10- Seleccionar la opción para contenido privado (símbolo de candado)   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">se visualiza el contenido privado del usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario accede a la vista previa de cada uno de los videos configurados con los ajustes de privacidad en modo “Sólo yo”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eliminar contenido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- seleccionar una publicación creada; 4- Seleccionar la opción “Más” (símbolo “...”; 5- Seleccionar la opción “Eliminar” (símbolo cesto de basura); 6- Confirmar la eliminación del contenido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El contenido es eliminado de la cuenta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La publicación es eliminada del listado de vistas previas de los contenidos creados por el usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seguir usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción “Siguiendo”; 4- Seleccionar la opción “Seguir” en la cuenta de otro usuario del listado en pantalla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario comienza a incrementar la red de contactos en la plataforma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El botón “Seguir” cambia de color y leyenda a “Siguiendo”. El contador de perfiles seguidos aumenta (de 0 a 1).</t>
   </si>
 </sst>
 </file>
@@ -843,7 +954,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.76"/>
@@ -1309,9 +1420,28 @@
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+    <row r="16" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -1319,29 +1449,59 @@
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+    <row r="17" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
+      <c r="K17" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+    <row r="18" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -1349,14 +1509,28 @@
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+    <row r="19" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>113</v>
+      </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1364,14 +1538,28 @@
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+    <row r="20" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -1379,14 +1567,26 @@
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
+    <row r="21" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="E21" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>123</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1394,14 +1594,26 @@
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
+    <row r="22" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="E22" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -1544,6 +1756,136 @@
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
     </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId2" display="breru.socio@gmail.com"/>
@@ -1558,6 +1900,11 @@
     <hyperlink ref="D13" r:id="rId11" display="breru.qatest@gmail.com"/>
     <hyperlink ref="D14" r:id="rId12" display="breru.qatest@gmail.com"/>
     <hyperlink ref="D15" r:id="rId13" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D16" r:id="rId14" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D17" r:id="rId15" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D18" r:id="rId16" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D19" r:id="rId17" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D20" r:id="rId18" display="breru.qatest@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1566,6 +1913,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId14"/>
+  <legacyDrawing r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Agregué casos de prueba de componente para la edición del perfil de usuario
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="210">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -91,10 +91,10 @@
     <t xml:space="preserve">Observaciones</t>
   </si>
   <si>
-    <t xml:space="preserve">cp₁</t>
-  </si>
-  <si>
-    <t xml:space="preserve">publicar sin registrar</t>
+    <t xml:space="preserve">CP-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realizar una publicación sin ser usuario registrado</t>
   </si>
   <si>
     <t xml:space="preserve">usuario sin registrar</t>
@@ -109,16 +109,22 @@
     <t xml:space="preserve">No permite realizar ninguna publicación hasta que el usuario cree su propia cuenta</t>
   </si>
   <si>
-    <t xml:space="preserve">Permite realizar todos los pasos de creación de una publicación. No permite finalizar la misma hasta que el usuario esté Registrado</t>
+    <t xml:space="preserve">Permite realizar todos los pasos de creación de una publicación pero no permite finalizar la misma hasta que el usuario esté Registrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta</t>
   </si>
   <si>
     <t xml:space="preserve">La aplicación no guarda la publicación creada como “Borrador” durante el proceso de registro, lo cual obliga al usuario a volver a crearla, editarla y repetir todos los pasos nuevamente.   </t>
   </si>
   <si>
-    <t xml:space="preserve">cp-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registro exitoso con credenciales correctas</t>
+    <t xml:space="preserve">CP-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar Registro exitoso con credenciales correctas</t>
   </si>
   <si>
     <t xml:space="preserve">Email: breru.socio@gmail.com; Contraseña: tiktok123//</t>
@@ -136,7 +142,7 @@
     <t xml:space="preserve">cp3</t>
   </si>
   <si>
-    <t xml:space="preserve">Registro con  email inválido</t>
+    <t xml:space="preserve">Validar rechazo de Registro con  email inválido</t>
   </si>
   <si>
     <t xml:space="preserve">Email: correo.com</t>
@@ -157,7 +163,7 @@
     <t xml:space="preserve">cp4</t>
   </si>
   <si>
-    <t xml:space="preserve">Registro con contraseña menor al límite inferior (7)</t>
+    <t xml:space="preserve">Validar rechazo de Registro con contraseña con cantidad de caracteres menor al límite inferior (7)</t>
   </si>
   <si>
     <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: tt1234/</t>
@@ -169,10 +175,31 @@
     <t xml:space="preserve">Se visualiza una tilde verde para la condición “Letras, números y caracteres especiales” pero no para la condición “Entre 8 y 20 caracteres”. No permite seleccionar la opción “Siguiente”.</t>
   </si>
   <si>
+    <t xml:space="preserve">Media</t>
+  </si>
+  <si>
     <t xml:space="preserve">cp5</t>
   </si>
   <si>
-    <t xml:space="preserve">Registro con contraseña mayor al límite superior (21)</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Validar rechazo de Registro con contraseña con cantidad de caracteres</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> mayor al límite superior (21)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: a234567891011121314**</t>
@@ -184,7 +211,7 @@
     <t xml:space="preserve">cp6</t>
   </si>
   <si>
-    <t xml:space="preserve">Registro con contraseña sin letra</t>
+    <t xml:space="preserve">Validar rechazo de Registro con contraseña sin letra</t>
   </si>
   <si>
     <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: 1234567#</t>
@@ -246,7 +273,7 @@
     <t xml:space="preserve">cp7</t>
   </si>
   <si>
-    <t xml:space="preserve">Registro con contraseña sin número</t>
+    <t xml:space="preserve">Validar rechazo de Registro con contraseña sin número</t>
   </si>
   <si>
     <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: abcdefg$</t>
@@ -258,7 +285,25 @@
     <t xml:space="preserve">cp8</t>
   </si>
   <si>
-    <t xml:space="preserve">Registro con contraseña sin caracteres especiales</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Validar rechazo de </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Registro con contraseña sin caracteres especiales</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Email: ejemplo@prueba.com; Contraseña: a2345678</t>
@@ -270,7 +315,7 @@
     <t xml:space="preserve">cp9</t>
   </si>
   <si>
-    <t xml:space="preserve">error contraseña 1er intento</t>
+    <t xml:space="preserve">Login fallido por contraseña incorrecta: 1er intento. Validar que el usuario se mantenga en estado Logged Out con 6 intentos más</t>
   </si>
   <si>
     <t xml:space="preserve">usuario registrado en estado logged out</t>
@@ -309,7 +354,7 @@
     <t xml:space="preserve">cp10</t>
   </si>
   <si>
-    <t xml:space="preserve">error contraseña 2do intento</t>
+    <t xml:space="preserve">Login fallido por contraseña incorrecta: 2do intento. Validar que el usuario se mantenga en estado Logged Out con 5 intentos más</t>
   </si>
   <si>
     <r>
@@ -349,7 +394,7 @@
     <t xml:space="preserve">cp11</t>
   </si>
   <si>
-    <t xml:space="preserve">error contraseña supera número máximo de intentos (7)</t>
+    <t xml:space="preserve">Login fallido por contraseña incorrecta: 7mo intento. Validar que el usuario pase al estado Blocked una vez superado el límite de intentos</t>
   </si>
   <si>
     <r>
@@ -386,7 +431,7 @@
     <t xml:space="preserve">Aviso de contraseña incorrecta. El usuario pasa al estado blocked</t>
   </si>
   <si>
-    <t xml:space="preserve">se visualiza la leyenda “Has superado el límite de intentos para introducir la cuenta o la contraseña. Inténtalo de nuevo en 30 mm.”</t>
+    <t xml:space="preserve">Se visualiza la leyenda “Has superado el límite de intentos para introducir la cuenta o la contraseña. Inténtalo de nuevo en 30 mm.”</t>
   </si>
   <si>
     <t xml:space="preserve">A medida que se realizan los intentos fallidos, se visualiza una cuenta regresiva que indica la cantidad de intentos restantes.</t>
@@ -395,7 +440,7 @@
     <t xml:space="preserve">cp12</t>
   </si>
   <si>
-    <t xml:space="preserve">Inicio de sesión de usuario en estado blocked antes de completar el tiempo de espera para nuevos intentos</t>
+    <t xml:space="preserve">Validar rechazo de Inicio de sesión de usuario en estado Blocked antes de completar el tiempo de espera para nuevos intentos</t>
   </si>
   <si>
     <t xml:space="preserve">usuario en estado blocked</t>
@@ -444,7 +489,7 @@
     <t xml:space="preserve">cp13</t>
   </si>
   <si>
-    <t xml:space="preserve">Restablecer contraseña</t>
+    <t xml:space="preserve">Validar que el usuario pueda Restablecer contraseña</t>
   </si>
   <si>
     <t xml:space="preserve">Email: breru.qatest@gmail.com</t>
@@ -560,7 +605,7 @@
     <t xml:space="preserve">cp15</t>
   </si>
   <si>
-    <t xml:space="preserve">compartir video</t>
+    <t xml:space="preserve">Compartir video exitosamente</t>
   </si>
   <si>
     <t xml:space="preserve">usuario en estado logged in </t>
@@ -569,7 +614,7 @@
     <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Compartir” (símbolo flecha); 4- Seleccionar la aplicación WhatsApp; 5- Seleccionar un contacto; 6- Enviar</t>
   </si>
   <si>
-    <t xml:space="preserve">el sistema permite compartir el video en diferentes redes sociales, entre ella WhatsApp</t>
+    <t xml:space="preserve">El sistema permite compartir el video en diferentes redes sociales, entre ellas WhatsApp</t>
   </si>
   <si>
     <t xml:space="preserve">Se visualizan los íconos de las diferentes aplicaciones a las que se puede compartir el contenido. Permite seleccionar contactos y enviar por WhatsApp </t>
@@ -578,16 +623,16 @@
     <t xml:space="preserve">cp16</t>
   </si>
   <si>
-    <t xml:space="preserve">dejar comentarios</t>
+    <t xml:space="preserve">Comentar video exitosamente</t>
   </si>
   <si>
     <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Comentar” (símbolo globo de diálogo); 4- Ingresar un comentario en el campo “Añadir comentario”; 5- Enviar</t>
   </si>
   <si>
-    <t xml:space="preserve">el sistema permite añadir un comentario a la publicación seleccionada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Al ingresar a los comentarios, se visualiza el último comentario agregado primero en la lista (orden: intercalados entre sí, con diferentes tiempos de realización)</t>
+    <t xml:space="preserve">El sistema permite añadir un comentario a la publicación seleccionada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario puede comentar el video. Al ingresar a la sección de los comentarios, se visualiza el más actual  primero en la lista (orden: intercalados entre sí, con diferentes tiempos de realización)</t>
   </si>
   <si>
     <t xml:space="preserve">Al actualizar la pantalla e ingresar nuevamente al listado de comentarios de la publicación, cambia el orden de la lista. El último comentario realizado aparece al final (orden: del más antiguo al menos antiguo)</t>
@@ -596,7 +641,7 @@
     <t xml:space="preserve">cp17</t>
   </si>
   <si>
-    <t xml:space="preserve">guardar contenido</t>
+    <t xml:space="preserve">Guardar contenido exitosamente</t>
   </si>
   <si>
     <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Guardar” (símbolo de marcador); 4- Ingresar al perfil de usuario; 5- seleccionar mismo símbolo de marcador</t>
@@ -611,13 +656,13 @@
     <t xml:space="preserve">cp18</t>
   </si>
   <si>
-    <t xml:space="preserve">visualizar Likes</t>
+    <t xml:space="preserve">Visualizar contenido al que se le dio “Like” exitosamente</t>
   </si>
   <si>
     <t xml:space="preserve">1- Iniciar sesión; 2- visualizar contenido generado por otra cuenta; 3- seleccionar la opción “Me gusta” (símbolo de corazón); 4- Ingresar al perfil de usuario; 5- seleccionar mismo símbolo </t>
   </si>
   <si>
-    <t xml:space="preserve">se visualiza el contenido “likeado”</t>
+    <t xml:space="preserve">Se visualiza el contenido “likeado”</t>
   </si>
   <si>
     <t xml:space="preserve">El usuario accede a la vista previa de cada uno de los videos a los que le dio Like</t>
@@ -626,13 +671,13 @@
     <t xml:space="preserve">cp19</t>
   </si>
   <si>
-    <t xml:space="preserve">crear contenido privado</t>
+    <t xml:space="preserve">Crear contenido de visualización privada para el usuario</t>
   </si>
   <si>
     <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- seleccionar la opción “Nuevo video” (símbolo “+”); 4- Seleccionar Cámara; 5- Crear publicación; 6- Seleccionar “Siguiente”; 7- Cambiar el ajuste de privacidad a “Sólo yo”; 8- Publicar; 9- Ingresar nuevamente al perfil; 10- Seleccionar la opción para contenido privado (símbolo de candado)   </t>
   </si>
   <si>
-    <t xml:space="preserve">se visualiza el contenido privado del usuario</t>
+    <t xml:space="preserve">Se visualiza el contenido privado del usuario</t>
   </si>
   <si>
     <t xml:space="preserve">El usuario accede a la vista previa de cada uno de los videos configurados con los ajustes de privacidad en modo “Sólo yo”</t>
@@ -641,7 +686,7 @@
     <t xml:space="preserve">cp20</t>
   </si>
   <si>
-    <t xml:space="preserve">eliminar contenido</t>
+    <t xml:space="preserve">Eliminar contenido exitosamente</t>
   </si>
   <si>
     <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- seleccionar una publicación creada; 4- Seleccionar la opción “Más” (símbolo “...”; 5- Seleccionar la opción “Eliminar” (símbolo cesto de basura); 6- Confirmar la eliminación del contenido</t>
@@ -656,7 +701,7 @@
     <t xml:space="preserve">cp21</t>
   </si>
   <si>
-    <t xml:space="preserve">seguir usuario</t>
+    <t xml:space="preserve">Seguir a otros usuarios</t>
   </si>
   <si>
     <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción “Siguiendo”; 4- Seleccionar la opción “Seguir” en la cuenta de otro usuario del listado en pantalla</t>
@@ -666,6 +711,556 @@
   </si>
   <si>
     <t xml:space="preserve">El botón “Seguir” cambia de color y leyenda a “Siguiendo”. El contador de perfiles seguidos aumenta (de 0 a 1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Añadir descripción en el perfil del usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción “+ Añadir descripción corta”; 4- Ingresar una descripción; 5- Seleccionar “Guardar” </t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario detalla una descripción de su bio para otros usuarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualiza la descripción realizada por el usuario en su perfil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar error por campo Nombre de perfil: vacío</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: (vacío)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Dejar el campo “Nombre de perfil” vacío </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La aplicación no permite continuar con la edición hasta completar el campo Nombre con al menos un carácter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El botón “Guardar” queda bloqueado y en color gris mientras el campo Nombre se encuentra vacío. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si el usuario no quiere editar su nombre de perfil, puede omitir esta acción, y el nombre queda asignado por defecto (user1019917313611)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar Nombre de perfil con mayúscula</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: Brenda</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”; 5- Seleccionar “Guardar”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario visualiza la leyenda con los requisitos válidos para el campo Nombre (hasta 30 caracteres). El botón “Guardar” queda bloqueado y en color gris hasta que el usuario ingresa el primer carácter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permite el ingreso de letra mayúscula sin visualizar un aviso de requisitos de validación para el campo Nombre respecto a el tipo de caracteres ingresados. El botón “Guardar” queda habilitado y en color rojo desde que el usuario ingresa el primer carácter, independientemente de cuál sea éste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar Nombre de perfil con números</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: 1234567</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Permite el ingreso de números </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">sin visualizar un aviso de requisitos de validación para el campo Nombre respecto a el tipo de caracteres ingresados. El botón “Guardar” queda habilitado y en color rojo desde que el usuario ingresa el primer carácter, independientemente de cuál sea éste</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">cp26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar Nombre de perfil con caracteres especiales</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: $%^)&gt;/</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Permite el ingreso de caracteres especiales </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">sin visualizar un aviso de requisitos de validación para el campo Nombre respecto a el tipo de caracteres ingresados. El botón “Guardar” queda habilitado y en color rojo desde que el usuario ingresa el primer carácter, independientemente de cuál sea éste</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">cp27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar Nombre de perfil con combinación de caracteres</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: Br-06^</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Permite el ingreso de cualquier carácter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar rechazo de Nombre de perfil &gt;30 caracteres (31)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: abcdefghijklmnñopqrstuvwxyz1234</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema rechaza el ingreso de 31 caracteres para el campo Nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El contador de caracteres debajo del campo Nombre incrementa. Al llegar a 30, se colorea en rojo y el sistema no permite ingresar más caracteres en el campo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Límite de intentos de edición del Nombre de perfil (1 vez cada 7 días)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Iniciar sesión; 2- Ingresar al perfil del usuario; 3- Seleccionar la opción para editar perfil (símbolo lápiz); 4- Completar el campo “Nombre de perfil”; 5- Seleccionar “Guardar”; 6- Seleccionar “Continuar”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema acepta el formato ingresado y bloquea el campo Nombre durante 7 días</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasadas las 24hs de establecido el Nombre de Perfil, el sistema volvió a habilitar la edición del mismo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No pasa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG: esto se observó manteniendo la app funcionando en segundo plano en el dispositivo movil (Samsung A56), sin apagar ni reiniciar el equipo. Pasadas las 24hs, cuando se volvió a ingresar a la app desde la vista previa de aplicaciones ejecutadas en segundo plano, la pantalla mostró nuevamente el campo Nombre de Perfil con el nombre prestablecido al crear la cuenta nueva.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar el rechazo de Nombre de usuario con  formato incorrecto: 1 carácter; mayúscula</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: B</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema rechaza los datos ingresados por incumplimiento de requisitos: al menos dos caracteres, sin mayúsculas</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Aparece una leyenda que indica que el nombre debe contener al menos 2 caracteres, pero no hace mención al uso de mayúsculas.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> El botón “Guardar” queda bloqueado y en color gris.  Las opciones del usuario son: probar nuevamente u omitir la edición</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG: el rechazo es validado únicamente por ser &lt;2 caracteres, sin especificar que el uso de mayúscula es inválido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar el rechazo de Nombre de usuario con  formato incorrecto: 2 caracteres siendo 1 mayúscula y 1 minúscula</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: Br</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema rechaza los datos ingresados y se visualiza una leyenda con los requisitos válidos para el campo Nombre</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">El sistema rechaza los datos ingresados, especificando cuáles son los requisitos válidos. El botón “Guardar” queda bloqueado y en color gris. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Las opciones del usuario son: probar nuevamente u omitir la edición</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">A partir del momento en que se ingresaron 2 (dos) caracteres, el usuario puede visualizar los requisitos: minúsculas, números, guiones bajos y puntos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar el rechazo de Nombre de usuario con formato incorrecto: caracteres especiales inválidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema no acepta el formato ingresado. Se visualiza una leyenda con los requisitos válidos </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">El sistema rechaza el formato ingresado y se visualiza una leyenda con los requisitos válidos (minúsculas, números, guiones bajos y puntos).</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> El botón “Guardar” queda bloqueado y en color gris.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Las opciones del usuario son: probar nuevamente u omitir la edición</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">cp33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar rechazo del Nombre de usuario cuando finaliza en “.”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: br06.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema rechaza los datos ingresados y se visualiza una leyenda indicando que el Nombre de usuario no puede terminar con “.”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp34</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Validar </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Nombre de usuario cuando finaliza en número</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: br06.4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">El sistema acepta el formato ingresado </t>
+  </si>
+  <si>
+    <t xml:space="preserve">El usuario visualiza una tilde verde que indica que el formato del Nombre es correcto. El botón “Guardar” queda habilitado y en color rojo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar Nombre de usuario cuando finaliza en “_”</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Email: breru.qatest@gmail.com; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Contraseña: tiktok123//; Nombre: br06._</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Una vez seleccionado “Guardar” aparece un cartel para confirmar el nombre de usuario, con un aviso restrictivo de modificación del mismo por 30 días.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cp36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ejecución en segundo plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1- Ingresar a la app; 2- Dejarla ejecutándose en 2do plano; 3- Ingresar a otra pantalla del dispositivo (Ej: Ajustes); 4- Tocar el botón para visualizar las apps abiertas en 2do plano (símbolo de 3 rayas verticales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se visualiza la app junto con otras pantallas en 2do plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La vista previa de la app en 2do plano desaparece. Se requiere volver a abrir la app nuevamente, ya sea desde el menú de aplicaciones del dispositivo o desde el acceso directo a las últimas aplicaciones utilizadas</t>
   </si>
 </sst>
 </file>
@@ -752,7 +1347,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -762,6 +1357,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -954,7 +1553,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.76"/>
@@ -1026,813 +1625,1255 @@
       <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K2" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K4" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
+        <v>38</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="J6" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="87" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
+        <v>63</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="97.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="108.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K12" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="108.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K13" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K14" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" customFormat="false" ht="184.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="161.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
+        <v>94</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
+        <v>100</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
+        <v>105</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K17" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
+        <v>116</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="151.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
+        <v>121</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" customFormat="false" ht="161.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="97.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D21" s="2"/>
+        <v>97</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="E21" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
+        <v>126</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="76.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>97</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="E22" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
+        <v>131</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
+    <row r="23" customFormat="false" ht="65.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
+    <row r="24" customFormat="false" ht="69.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>143</v>
+      </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+    <row r="25" customFormat="false" ht="138.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+    <row r="26" customFormat="false" ht="129.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
+    <row r="27" customFormat="false" ht="140.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
+    <row r="28" customFormat="false" ht="97.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+    <row r="29" customFormat="false" ht="76.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>168</v>
+      </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
+    <row r="30" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>175</v>
+      </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
+    <row r="31" customFormat="false" ht="119.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>181</v>
+      </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+    <row r="32" customFormat="false" ht="108.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="119.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K33" s="2"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="65.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K34" s="2"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="65.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="K35" s="2"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="65.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>206</v>
+      </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
+      <c r="E37" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>209</v>
+      </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2"/>
@@ -1846,6 +2887,8 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2"/>
@@ -1859,6 +2902,8 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
@@ -1885,6 +2930,110 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1905,6 +3054,22 @@
     <hyperlink ref="D18" r:id="rId16" display="breru.qatest@gmail.com"/>
     <hyperlink ref="D19" r:id="rId17" display="breru.qatest@gmail.com"/>
     <hyperlink ref="D20" r:id="rId18" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D21" r:id="rId19" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D22" r:id="rId20" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D23" r:id="rId21" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D24" r:id="rId22" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D25" r:id="rId23" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D26" r:id="rId24" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D27" r:id="rId25" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D28" r:id="rId26" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D29" r:id="rId27" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D30" r:id="rId28" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D31" r:id="rId29" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D32" r:id="rId30" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D33" r:id="rId31" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D34" r:id="rId32" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D35" r:id="rId33" display="breru.qatest@gmail.com"/>
+    <hyperlink ref="D36" r:id="rId34" display="breru.qatest@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1913,6 +3078,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId19"/>
+  <legacyDrawing r:id="rId35"/>
 </worksheet>
 </file>
</xml_diff>